<commit_message>
Retention v2: 22–30 s Shorts, frame-0 hooks, anime power-up FX
Week-one analytics (37.4% stayed, 62.6% swiped, ~1K ceiling) showed the best
moment arriving at 10–15 s. Rewrites the hooks and beat sheets for V013–V035
and every unproduced hack (plan/retention_v2.py → retention_v2.csv, both plan
CSVs and the plan xlsx), queues a V013 re-cut, and adds shared/powerup.tsx:
generic anime-style hook presets (charge, impact, beam, dash, clash, meter)
with a PowerUpDemo reference composition. PIPELINE §5 and WRITING §G updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015PViZ5ubA2qW6NZd7JkSHQ
</commit_message>
<xml_diff>
--- a/plan/Stickman_Shorts_Content_Plan.xlsx
+++ b/plan/Stickman_Shorts_Content_Plan.xlsx
@@ -1894,12 +1894,12 @@
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>AI WON'T TAKE YOUR JOB…</t>
+          <t>AI USERS: −19 POINTS</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>‘AI won't take your job, someone using AI will.’ Half true.</t>
+          <t>These consultants used GPT-4 and got nineteen points worse.</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1924,11 +1924,11 @@
       </c>
       <c r="N14" s="4" t="inlineStr">
         <is>
-          <t>Boss walks in again</t>
+          <t>'Because the next report—' → cut to the crashing bar</t>
         </is>
       </c>
       <c r="O14" s="4" t="n">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="P14" s="4" t="inlineStr">
         <is>
@@ -1990,12 +1990,12 @@
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>₹0. BETTER LUCK NEXT TIME.</t>
+          <t>₹0. AGAIN.</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>Why does a payment app hand you a scratch card that's usually empty?</t>
+          <t>You've scratched a hundred of these and won almost nothing.</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -2020,11 +2020,11 @@
       </c>
       <c r="N15" s="4" t="inlineStr">
         <is>
-          <t>Scratch card reappears</t>
+          <t>'Now scratch—' → first card again</t>
         </is>
       </c>
       <c r="O15" s="4" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="P15" s="4" t="inlineStr">
         <is>
@@ -2086,12 +2086,12 @@
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>👍</t>
+          <t>HE BUILT 👍. THEN BLOCKED IT.</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>One of the people who helped build the Like button now limits his own apps.</t>
+          <t>He helped build the Like button. Then locked it out of his own phone.</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
@@ -2116,11 +2116,11 @@
       </c>
       <c r="N16" s="4" t="inlineStr">
         <is>
-          <t>Thumb shrinks</t>
+          <t>'Because the next like—' → thumb grows again</t>
         </is>
       </c>
       <c r="O16" s="4" t="n">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="P16" s="4" t="inlineStr">
         <is>
@@ -2182,12 +2182,12 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>ESTIMATE: 2 DAYS</t>
+          <t>ESTIMATE: 2 DAYS. ACTUAL: ?</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>Your estimate: 2 days. Reality: 2 weeks. Why is it always this?</t>
+          <t>You said two days. It's been two weeks.</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -2212,11 +2212,11 @@
       </c>
       <c r="N17" s="4" t="inlineStr">
         <is>
-          <t>Calendar resets</t>
+          <t>'Now, how long for—' → stamp again</t>
         </is>
       </c>
       <c r="O17" s="4" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="P17" s="4" t="inlineStr">
         <is>
@@ -2278,12 +2278,12 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>~₹2,999~ ₹999</t>
+          <t>₹2,999 ✗  ₹999 = STEAL?</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>Myth: the crossed-out price tells you what it's worth.</t>
+          <t>That crossed-out ₹2,999 was never the price. It's bait.</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -2308,11 +2308,11 @@
       </c>
       <c r="N18" s="4" t="inlineStr">
         <is>
-          <t>Anchor drops again</t>
+          <t>'Now look at the next—' → anchor drops</t>
         </is>
       </c>
       <c r="O18" s="4" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="P18" s="4" t="inlineStr">
         <is>
@@ -2379,7 +2379,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>Typing… stopped. Typing… stopped. Why does this hurt so much?</t>
+          <t>Typing. Stopped. Typing. Stopped. Why is this torture?</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -2404,11 +2404,11 @@
       </c>
       <c r="N19" s="4" t="inlineStr">
         <is>
-          <t>Dots start again</t>
+          <t>'Oh, they're typing—' → dots again</t>
         </is>
       </c>
       <c r="O19" s="4" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="P19" s="4" t="inlineStr">
         <is>
@@ -2475,7 +2475,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>AI doesn't lie to you. It does something weirder.</t>
+          <t>It answered instantly. Confidently. And it was completely wrong.</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -2500,11 +2500,11 @@
       </c>
       <c r="N20" s="4" t="inlineStr">
         <is>
-          <t>Actor bows</t>
+          <t>'Then ask it again—' → robot answers</t>
         </is>
       </c>
       <c r="O20" s="4" t="n">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="P20" s="4" t="inlineStr">
         <is>
@@ -2571,7 +2571,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>POV: the only way to close the pop-up is to insult yourself.</t>
+          <t>To close this pop-up, you have to insult yourself.</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -2596,11 +2596,11 @@
       </c>
       <c r="N21" s="4" t="inlineStr">
         <is>
-          <t>Pop-up returns</t>
+          <t>'Click no. Then—' → pop-up returns</t>
         </is>
       </c>
       <c r="O21" s="4" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="P21" s="4" t="inlineStr">
         <is>
@@ -2667,7 +2667,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>Losing ₹500 hurts more than finding ₹500 feels good. How much more?</t>
+          <t>Losing five hundred rupees hurts more than finding it feels good.</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -2692,11 +2692,11 @@
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Scale tips again</t>
+          <t>'So next time you—' → the two notes again</t>
         </is>
       </c>
       <c r="O22" s="4" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="P22" s="4" t="inlineStr">
         <is>
@@ -2763,7 +2763,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>POV: AI wrote 500 lines and you reviewed five.</t>
+          <t>AI wrote five hundred lines. You reviewed five.</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -2788,11 +2788,11 @@
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>LGTM again</t>
+          <t>'LGTM—' → scroll drops again</t>
         </is>
       </c>
       <c r="O23" s="4" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="P23" s="4" t="inlineStr">
         <is>
@@ -2854,7 +2854,7 @@
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>FAILED.</t>
+          <t>THIS GLUE FAILED.</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
@@ -2884,11 +2884,11 @@
       </c>
       <c r="N24" s="4" t="inlineStr">
         <is>
-          <t>Note sticks</t>
+          <t>'So keep your failures, because—' → stamp again</t>
         </is>
       </c>
       <c r="O24" s="4" t="n">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="P24" s="4" t="inlineStr">
         <is>
@@ -2955,7 +2955,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>You didn't like it. You didn't comment. The algorithm still knows you wanted it.</t>
+          <t>You didn't like it. You didn't comment. It still knows.</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -2980,11 +2980,11 @@
       </c>
       <c r="N25" s="4" t="inlineStr">
         <is>
-          <t>Clerk clicks the stopwatch again</t>
+          <t>'Click—' → stopwatch again</t>
         </is>
       </c>
       <c r="O25" s="4" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="P25" s="4" t="inlineStr">
         <is>
@@ -3051,7 +3051,7 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>POV: the movie is terrible but you paid ₹400, so you stay.</t>
+          <t>The movie is terrible, but you paid four hundred, so you stay.</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -3076,11 +3076,11 @@
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Credits roll</t>
+          <t>'Credits roll—' → back in the seat</t>
         </is>
       </c>
       <c r="O26" s="4" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="P26" s="4" t="inlineStr">
         <is>
@@ -3142,12 +3142,12 @@
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>ONLY 2 LEFT IN STOCK!</t>
+          <t>ONLY 2 LEFT!</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>‘Only 2 left.’ Are there really only two?</t>
+          <t>Only two left. Are there really only two?</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -3172,11 +3172,11 @@
       </c>
       <c r="N27" s="4" t="inlineStr">
         <is>
-          <t>Timer resets to 10:00</t>
+          <t>'Timer resets to 10:00—' → slam again</t>
         </is>
       </c>
       <c r="O27" s="4" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="P27" s="4" t="inlineStr">
         <is>
@@ -3238,12 +3238,12 @@
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>MAKE IT BETTER.</t>
+          <t>MAKE IT BETTER. (×47)</t>
         </is>
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>POV: you've typed 'make it better' 47 times.</t>
+          <t>You've typed 'make it better' forty-seven times.</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -3268,11 +3268,11 @@
       </c>
       <c r="N28" s="4" t="inlineStr">
         <is>
-          <t>Wheel spins</t>
+          <t>'Make it better—' → wheel spins</t>
         </is>
       </c>
       <c r="O28" s="4" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="P28" s="4" t="inlineStr">
         <is>
@@ -3339,7 +3339,7 @@
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Myth: cab apps raise prices when your battery is low.</t>
+          <t>Does your cab price go up when your battery is low?</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -3364,11 +3364,11 @@
       </c>
       <c r="N29" s="4" t="inlineStr">
         <is>
-          <t>Battery icon blinks</t>
+          <t>'Battery blinks—' → 4% again</t>
         </is>
       </c>
       <c r="O29" s="4" t="n">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="P29" s="4" t="inlineStr">
         <is>
@@ -3435,7 +3435,7 @@
       </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Most of what you watch on YouTube, you never searched for.</t>
+          <t>Most of what you watch, you never searched for.</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -3460,11 +3460,11 @@
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Counter returns to 70%</t>
+          <t>'Up next—' → conveyor again</t>
         </is>
       </c>
       <c r="O30" s="4" t="n">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="P30" s="4" t="inlineStr">
         <is>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>The microwave oven started with a melted chocolate bar.</t>
+          <t>The microwave started with a melted chocolate bar.</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -3556,11 +3556,11 @@
       </c>
       <c r="N31" s="4" t="inlineStr">
         <is>
-          <t>Chocolate melts again</t>
+          <t>'Melts again—' → beam</t>
         </is>
       </c>
       <c r="O31" s="4" t="n">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="P31" s="4" t="inlineStr">
         <is>
@@ -3627,7 +3627,7 @@
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>POV: the client wants one small change.</t>
+          <t>The client wants one small change.</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -3652,11 +3652,11 @@
       </c>
       <c r="N32" s="4" t="inlineStr">
         <is>
-          <t>Pebble returns</t>
+          <t>'One small change—' → pebble again</t>
         </is>
       </c>
       <c r="O32" s="4" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="P32" s="4" t="inlineStr">
         <is>
@@ -3718,12 +3718,12 @@
       </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>₹99</t>
+          <t>₹99 ≠ ₹100?</t>
         </is>
       </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>₹99 isn't ₹100. Your brain treats it like ₹90.</t>
+          <t>Ninety-nine rupees isn't a hundred. Your brain disagrees.</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -3748,7 +3748,7 @@
       </c>
       <c r="N33" s="4" t="inlineStr">
         <is>
-          <t>Keyhole closes</t>
+          <t>'Keyhole closes—' → ₹99 slams again</t>
         </is>
       </c>
       <c r="O33" s="4" t="n">
@@ -3814,12 +3814,12 @@
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>1 THUMB vs 1,000 EXPERIMENTS</t>
+          <t>1 THUMB vs 1,000 TESTS</t>
         </is>
       </c>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>It's not a fair fight. It's your willpower versus thousands of A/B tests.</t>
+          <t>It's your willpower against thousands of A/B tests.</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -3844,11 +3844,11 @@
       </c>
       <c r="N34" s="4" t="inlineStr">
         <is>
-          <t>Army regroups</t>
+          <t>'The army regroups—' → clash again</t>
         </is>
       </c>
       <c r="O34" s="4" t="n">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="P34" s="4" t="inlineStr">
         <is>
@@ -3915,7 +3915,7 @@
       </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>POV: you asked AI if your startup idea is good.</t>
+          <t>You asked AI if your startup idea is good.</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3940,11 +3940,11 @@
       </c>
       <c r="N35" s="4" t="inlineStr">
         <is>
-          <t>Pom-poms again</t>
+          <t>'Is my idea good—' → pom-poms</t>
         </is>
       </c>
       <c r="O35" s="4" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="P35" s="4" t="inlineStr">
         <is>
@@ -4006,12 +4006,12 @@
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>75% AUTO-REJECTED?</t>
+          <t>MYTH: 75% AUTO-REJECTED</t>
         </is>
       </c>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Myth: 75% of resumes are rejected by robots before a human sees them.</t>
+          <t>Seventy-five percent of resumes rejected by robots? Prove it.</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -4036,11 +4036,11 @@
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Badge falls off</t>
+          <t>'Badge falls off—' → beam</t>
         </is>
       </c>
       <c r="O36" s="4" t="n">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="P36" s="4" t="inlineStr">
         <is>

</xml_diff>